<commit_message>
Add reviewed tweets REVIEWED_StateRepHong_20210107_20210317_20260806_autoPush.xlsx
</commit_message>
<xml_diff>
--- a/reviews/REVIEWED_StateRepHong_20210107_20210317_20260806_autoPush.xlsx
+++ b/reviews/REVIEWED_StateRepHong_20210107_20210317_20260806_autoPush.xlsx
@@ -3470,7 +3470,7 @@
         <v>0</v>
       </c>
       <c r="J70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K70" t="inlineStr"/>
     </row>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="J71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="inlineStr"/>
     </row>
@@ -3556,7 +3556,7 @@
         <v>0</v>
       </c>
       <c r="J72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" t="inlineStr"/>
     </row>

</xml_diff>